<commit_message>
docs: release planning capacités pour 6 personnes
</commit_message>
<xml_diff>
--- a/IPSSI_APOCAL_KIT/docs/cadrage/05-release-planning.xlsx
+++ b/IPSSI_APOCAL_KIT/docs/cadrage/05-release-planning.xlsx
@@ -116,7 +116,7 @@
     <t xml:space="preserve">✅ BON</t>
   </si>
   <si>
-    <t xml:space="preserve">« Sprint 1 : Objectif = setup MVP F1 + F2 · Capacité 28 h-pers · Vélocité 10 SP · Stories US-01, US-02 »</t>
+    <t xml:space="preserve">« Sprint 1 : Objectif = setup MVP F1 + F2 · Capacité 24 h-pers · Vélocité 10 SP · Stories US-01, US-02 »</t>
   </si>
   <si>
     <t xml:space="preserve">❌ À ÉVITER</t>
@@ -446,7 +446,7 @@
     <t xml:space="preserve">9 lignes planifiées avec jour, horaires et capacités</t>
   </si>
   <si>
-    <t xml:space="preserve">L'équipe taille est explicite (ex. 7 personnes), pas de capacité "floue"</t>
+    <t xml:space="preserve">L'équipe taille est explicite (ex. 6 personnes), pas de capacité "floue"</t>
   </si>
   <si>
     <t xml:space="preserve">6 personnes, capacités recalculées (174 h-pers)</t>

</xml_diff>